<commit_message>
monthly commission rate. If a monthly commission rate is set, it will be displayed in a prominent blue badge; otherwise, the default commission rate will be shown in a muted gray text.
</commit_message>
<xml_diff>
--- a/outputs/Payroll_Summary_2025-10.xlsx
+++ b/outputs/Payroll_Summary_2025-10.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,65 +436,70 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>全名</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>工時</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>OT工時</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>底薪</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>總佣金</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>津貼</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>報銷</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>微調</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>出勤獎</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>總收入</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>MPF扣除</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MPF狀態</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>實發薪資</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>地點</t>
         </is>
@@ -506,21 +511,23 @@
           <t>Carol</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Yuen Maria Wing Yan</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>42</v>
       </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
       <c r="D2" t="n">
-        <v>2730</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
+        <v>2520</v>
+      </c>
+      <c r="F2" t="n">
         <v>1997.46</v>
       </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
@@ -531,20 +538,23 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>4727.46</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="inlineStr">
+        <v>4517.46</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M2" t="n">
-        <v>4727.46</v>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" t="n">
+        <v>4517.46</v>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>Suning TKO Roadshow</t>
         </is>
@@ -556,21 +566,23 @@
           <t>Irene</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chan Yun Hing</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>204</v>
       </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
       <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
         <v>12240</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>7834.96</v>
       </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
@@ -581,20 +593,23 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
         <v>20074.96</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>20074.96</v>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>SW Wing On</t>
         </is>
@@ -606,21 +621,23 @@
           <t>Joe</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Wong Sui Ping</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>115</v>
       </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
       <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
         <v>6900</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>2220.58</v>
       </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
@@ -631,20 +648,23 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
         <v>9120.58</v>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>9120.58</v>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Tai Po Yata</t>
         </is>
@@ -656,21 +676,23 @@
           <t>Ling</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lok Yin Ling</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>105.5</v>
       </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
       <c r="D5" t="n">
-        <v>5802.5</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
+        <v>6330</v>
+      </c>
+      <c r="F5" t="n">
         <v>1604.05</v>
       </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
@@ -681,20 +703,23 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>7406.55</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="inlineStr">
+        <v>7934.05</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M5" t="n">
-        <v>7406.55</v>
-      </c>
-      <c r="N5" t="inlineStr">
+      <c r="N5" t="n">
+        <v>7934.05</v>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>Yuen Long Citistore</t>
         </is>
@@ -706,21 +731,23 @@
           <t>Mei Kiu</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Leung Mei Kiu</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>48</v>
       </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
       <c r="D6" t="n">
-        <v>3120</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
+        <v>2880</v>
+      </c>
+      <c r="F6" t="n">
         <v>121.92</v>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
@@ -731,20 +758,23 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>3241.92</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr">
+        <v>3001.92</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M6" t="n">
-        <v>3241.92</v>
-      </c>
-      <c r="N6" t="inlineStr">
+      <c r="N6" t="n">
+        <v>3001.92</v>
+      </c>
+      <c r="O6" t="inlineStr">
         <is>
           <t>Tuen Wan Aeon</t>
         </is>
@@ -756,45 +786,50 @@
           <t>Mei Kiu</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Leung Mei Kiu</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>48</v>
       </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
       <c r="D7" t="n">
-        <v>3120</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
+        <v>2880</v>
+      </c>
+      <c r="F7" t="n">
         <v>253.7</v>
       </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
       <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>30</v>
       </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>3403.7</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr">
+        <v>3163.7</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M7" t="n">
-        <v>3403.7</v>
-      </c>
-      <c r="N7" t="inlineStr">
+      <c r="N7" t="n">
+        <v>3163.7</v>
+      </c>
+      <c r="O7" t="inlineStr">
         <is>
           <t>Tuen Wan Yata</t>
         </is>
@@ -806,21 +841,23 @@
           <t>Pinky</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cheung Yin Ping</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>16</v>
       </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
       <c r="D8" t="n">
-        <v>1040</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
+        <v>960</v>
+      </c>
+      <c r="F8" t="n">
         <v>236.67</v>
       </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
@@ -831,20 +868,23 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1276.67</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
+        <v>1196.67</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M8" t="n">
-        <v>1276.67</v>
-      </c>
-      <c r="N8" t="inlineStr">
+      <c r="N8" t="n">
+        <v>1196.67</v>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>Tai Po Yata</t>
         </is>
@@ -856,24 +896,26 @@
           <t>Wah</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Lo Chun Wah</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>171</v>
       </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
       <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>10260</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>3591.57</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>630</v>
       </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
@@ -881,20 +923,23 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
         <v>14481.57</v>
       </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>14481.57</v>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Kowloon Bay Fortress</t>
         </is>
@@ -906,21 +951,23 @@
           <t>Wu Sir</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Woo Kin Ming</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>56</v>
       </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
       <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>3640</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>1542.3</v>
       </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
@@ -931,20 +978,23 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
         <v>5182.3</v>
       </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>5182.3</v>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Kwai Fong Fortress</t>
         </is>
@@ -956,21 +1006,23 @@
           <t>Yu</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Chan Fung Yu</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>32</v>
       </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
       <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
         <v>1920</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>277.32</v>
       </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
@@ -981,20 +1033,23 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
         <v>2197.32</v>
       </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="inlineStr">
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>🚫 永久豁免 (非 MPF 員工)</t>
         </is>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>2197.32</v>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Kwai Fong Fortress</t>
         </is>

</xml_diff>